<commit_message>
Invoice PDF: DH currency suffix, client address, EUR→MAD exchange rate
- Every amount on the invoice now carries its unit ("DH"/"EUR") in the
  value itself; the static "DH" boxes were removed from the template.
- The cell under the client name (B11) is now client_address, pre-filled
  from the client's saved address.
- Missions get an optional exchangeRate (EUR→MAD), shown in the
  create/edit forms only for EUR missions and cleared when switching to
  MAD. EUR invoices print a "Taux de change" line plus the Total TTC
  converted to MAD on a new template row 38 (hidden when no rate).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KmxYSmKMoDAecqgwkm1RPi
</commit_message>
<xml_diff>
--- a/backend/templates/invoice-template-default.xlsx
+++ b/backend/templates/invoice-template-default.xlsx
@@ -702,7 +702,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="129">
+  <cellXfs count="135">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1083,6 +1083,24 @@
     </xf>
     <xf numFmtId="0" fontId="30" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1902,9 +1920,7 @@
       </c>
       <c r="L20" s="59"/>
       <c r="M20" s="59"/>
-      <c r="N20" s="48" t="s">
-        <v>24</v>
-      </c>
+      <c r="N20" s="48"/>
       <c r="O20" s="49"/>
       <c r="P20" s="2"/>
     </row>
@@ -1975,9 +1991,7 @@
       </c>
       <c r="L23" s="70"/>
       <c r="M23" s="70"/>
-      <c r="N23" s="71" t="s">
-        <v>24</v>
-      </c>
+      <c r="N23" s="71"/>
       <c r="O23" s="72"/>
       <c r="P23" s="2"/>
     </row>
@@ -2135,9 +2149,7 @@
       </c>
       <c r="L31" s="108"/>
       <c r="M31" s="108"/>
-      <c r="N31" s="106" t="s">
-        <v>24</v>
-      </c>
+      <c r="N31" s="106"/>
       <c r="O31" s="109"/>
       <c r="P31" s="2"/>
       <c r="Q31" s="2"/>
@@ -2240,9 +2252,7 @@
       <c r="J36" s="120"/>
       <c r="K36" s="120"/>
       <c r="L36" s="120"/>
-      <c r="M36" s="121" t="s">
-        <v>24</v>
-      </c>
+      <c r="M36" s="121"/>
       <c r="N36" s="121"/>
       <c r="O36" s="122"/>
       <c r="P36" s="2"/>
@@ -2269,20 +2279,20 @@
     </row>
     <row r="38" ht="18" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
-      <c r="B38" s="2"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="2"/>
-      <c r="G38" s="2"/>
+      <c r="B38" s="129"/>
+      <c r="C38" s="130"/>
+      <c r="D38" s="130"/>
+      <c r="E38" s="130"/>
+      <c r="F38" s="130"/>
+      <c r="G38" s="131"/>
       <c r="H38" s="2"/>
-      <c r="I38" s="2"/>
-      <c r="J38" s="2"/>
-      <c r="K38" s="2"/>
-      <c r="L38" s="2"/>
-      <c r="M38" s="2"/>
-      <c r="N38" s="2"/>
-      <c r="O38" s="2"/>
+      <c r="I38" s="132"/>
+      <c r="J38" s="133"/>
+      <c r="K38" s="133"/>
+      <c r="L38" s="133"/>
+      <c r="M38" s="133"/>
+      <c r="N38" s="133"/>
+      <c r="O38" s="134"/>
       <c r="P38" s="2"/>
       <c r="Q38" s="2"/>
       <c r="R38" s="2"/>
@@ -2532,7 +2542,7 @@
       <c r="P51" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="62">
+  <mergeCells count="60">
     <mergeCell ref="A1:P6"/>
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="H8:J8"/>
@@ -2565,8 +2575,7 @@
     <mergeCell ref="D20:E20"/>
     <mergeCell ref="F20:H20"/>
     <mergeCell ref="I20:J20"/>
-    <mergeCell ref="K20:M20"/>
-    <mergeCell ref="N20:O20"/>
+    <mergeCell ref="K20:O20"/>
     <mergeCell ref="B22:E22"/>
     <mergeCell ref="F22:H22"/>
     <mergeCell ref="I22:J22"/>
@@ -2574,8 +2583,7 @@
     <mergeCell ref="B23:E24"/>
     <mergeCell ref="F23:H24"/>
     <mergeCell ref="I23:J24"/>
-    <mergeCell ref="K23:M24"/>
-    <mergeCell ref="N23:O24"/>
+    <mergeCell ref="K23:O24"/>
     <mergeCell ref="B25:E25"/>
     <mergeCell ref="F25:H25"/>
     <mergeCell ref="I25:J25"/>
@@ -2586,15 +2594,15 @@
     <mergeCell ref="I29:J30"/>
     <mergeCell ref="K29:O30"/>
     <mergeCell ref="I31:J31"/>
-    <mergeCell ref="K31:M31"/>
-    <mergeCell ref="N31:O31"/>
+    <mergeCell ref="K31:O31"/>
     <mergeCell ref="I34:O35"/>
     <mergeCell ref="B35:H35"/>
     <mergeCell ref="B36:G37"/>
-    <mergeCell ref="I36:L37"/>
-    <mergeCell ref="M36:O37"/>
+    <mergeCell ref="I36:O37"/>
     <mergeCell ref="B40:K41"/>
     <mergeCell ref="A43:P51"/>
+    <mergeCell ref="B38:G38"/>
+    <mergeCell ref="I38:O38"/>
   </mergeCells>
   <pageMargins left="0.2" right="0.2" top="0.25" bottom="0.25" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="56" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>